<commit_message>
feat: add SendToEmailPage component and configure API paths for email agent contacts
</commit_message>
<xml_diff>
--- a/public/email agent.xlsx
+++ b/public/email agent.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t xml:space="preserve">Email </t>
   </si>
@@ -28,12 +28,18 @@
     <t xml:space="preserve">Name </t>
   </si>
   <si>
+    <t xml:space="preserve">Type </t>
+  </si>
+  <si>
     <t xml:space="preserve">nitin.hackberrysoftech@gmail.com </t>
   </si>
   <si>
     <t xml:space="preserve">Nitin Mithapara</t>
   </si>
   <si>
+    <t xml:space="preserve">doctor email</t>
+  </si>
+  <si>
     <t xml:space="preserve">sachinhackberrysoftech@gmail.com </t>
   </si>
   <si>
@@ -44,6 +50,15 @@
   </si>
   <si>
     <t xml:space="preserve">Nirva Patel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pritmeghapara2516@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prit Meghapara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sponser</t>
   </si>
 </sst>
 </file>
@@ -126,16 +141,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -332,47 +351,72 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>7</v>
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="2"/>
+      <c r="C10" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A4" r:id="rId1" display="nirva.hackberry@gmail.com"/>
+    <hyperlink ref="A5" r:id="rId2" display="pritmeghapara2516@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>